<commit_message>
Fixed the translation not showing up on the home page
</commit_message>
<xml_diff>
--- a/translations/all-pages.xlsx
+++ b/translations/all-pages.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1815" uniqueCount="1362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1815" uniqueCount="1380">
   <si>
     <t>key</t>
   </si>
@@ -4108,6 +4108,60 @@
   </si>
   <si>
     <t>liveViewer.webSerialUnavailable</t>
+  </si>
+  <si>
+    <t>home.affiliation</t>
+  </si>
+  <si>
+    <t>home.brandHomeLabel</t>
+  </si>
+  <si>
+    <t>home.device.spod</t>
+  </si>
+  <si>
+    <t>home.device.tbd</t>
+  </si>
+  <si>
+    <t>home.device.ypod</t>
+  </si>
+  <si>
+    <t>home.device.ypodModified</t>
+  </si>
+  <si>
+    <t>home.page.browserTitle</t>
+  </si>
+  <si>
+    <t>home.page.eyebrow</t>
+  </si>
+  <si>
+    <t>Seletor das programas</t>
+  </si>
+  <si>
+    <t>home.page.title</t>
+  </si>
+  <si>
+    <t>home.program.aqiq</t>
+  </si>
+  <si>
+    <t>home.program.fireIq</t>
+  </si>
+  <si>
+    <t>home.program.sqiq</t>
+  </si>
+  <si>
+    <t>home.program.waterIq</t>
+  </si>
+  <si>
+    <t>home.program.waterIqUnavailableLabel</t>
+  </si>
+  <si>
+    <t>home.programs.ariaLabel</t>
+  </si>
+  <si>
+    <t>home.status.open</t>
+  </si>
+  <si>
+    <t>home.status.unavailable</t>
   </si>
 </sst>
 </file>
@@ -4978,15 +5032,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAE8341E-AA9D-44FB-828B-E8E7C198C373}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{AAE8341E-AA9D-44FB-828B-E8E7C198C373}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" ns3:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="27.6328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="49.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ns3:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5009,417 +5063,441 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>635</v>
-      </c>
-      <c r="B2" s="1" t="s">
+    <row r="2">
+      <c s="1" r="A2" t="s">
+        <v>1092</v>
+      </c>
+      <c s="1" r="B2" t="s">
         <v>636</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c s="1" r="C2" t="s">
         <v>637</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c s="1" r="D2" t="s">
+        <v>111</v>
+      </c>
+      <c s="1" r="E2" t="s">
+        <v>111</v>
+      </c>
+      <c s="1" r="F2" t="s">
+        <v>41</v>
+      </c>
+      <c s="1" r="G2" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="3">
+      <c s="1" r="A3" t="s">
+        <v>1094</v>
+      </c>
+      <c s="1" r="B3" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C3" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D3" t="s">
+        <v>114</v>
+      </c>
+      <c s="1" r="E3" t="s">
+        <v>114</v>
+      </c>
+      <c s="1" r="F3" t="s">
+        <v>115</v>
+      </c>
+      <c s="1" r="G3" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="4">
+      <c s="1" r="A4" t="s">
+        <v>1362</v>
+      </c>
+      <c s="1" r="B4" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C4" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D4" t="s">
+        <v>675</v>
+      </c>
+      <c s="1" r="E4" t="s">
+        <v>675</v>
+      </c>
+      <c s="1" r="F4" t="s">
+        <v>115</v>
+      </c>
+      <c s="1" r="G4" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="5">
+      <c s="1" r="A5" t="s">
+        <v>1363</v>
+      </c>
+      <c s="1" r="B5" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C5" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D5" t="s">
+        <v>646</v>
+      </c>
+      <c s="1" r="E5" t="s">
+        <v>881</v>
+      </c>
+      <c s="1" r="F5" t="s">
+        <v>647</v>
+      </c>
+      <c s="1" r="G5" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="6">
+      <c s="1" r="A6" t="s">
+        <v>1364</v>
+      </c>
+      <c s="1" r="B6" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C6" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D6" t="s">
+        <v>666</v>
+      </c>
+      <c s="1" r="E6" t="s">
+        <v>666</v>
+      </c>
+      <c s="1" r="F6" t="s">
+        <v>115</v>
+      </c>
+      <c s="1" r="G6" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="7">
+      <c s="1" r="A7" t="s">
+        <v>1365</v>
+      </c>
+      <c s="1" r="B7" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C7" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D7" t="s">
+        <v>672</v>
+      </c>
+      <c s="1" r="E7" t="s">
+        <v>672</v>
+      </c>
+      <c s="1" r="F7" t="s">
+        <v>115</v>
+      </c>
+      <c s="1" r="G7" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="8">
+      <c s="1" r="A8" t="s">
+        <v>1366</v>
+      </c>
+      <c s="1" r="B8" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C8" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D8" t="s">
+        <v>687</v>
+      </c>
+      <c s="1" r="E8" t="s">
+        <v>687</v>
+      </c>
+      <c s="1" r="F8" t="s">
+        <v>115</v>
+      </c>
+      <c s="1" r="G8" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="9">
+      <c s="1" r="A9" t="s">
+        <v>1367</v>
+      </c>
+      <c s="1" r="B9" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C9" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D9" t="s">
+        <v>690</v>
+      </c>
+      <c s="1" r="E9" t="s">
+        <v>690</v>
+      </c>
+      <c s="1" r="F9" t="s">
+        <v>115</v>
+      </c>
+      <c s="1" r="G9" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="10">
+      <c s="1" r="A10" t="s">
+        <v>1368</v>
+      </c>
+      <c s="1" r="B10" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C10" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D10" t="s">
+        <v>649</v>
+      </c>
+      <c s="1" r="E10" t="s">
+        <v>882</v>
+      </c>
+      <c s="1" r="F10" t="s">
+        <v>36</v>
+      </c>
+      <c s="1" r="G10" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="11">
+      <c s="1" r="A11" t="s">
+        <v>1369</v>
+      </c>
+      <c s="1" r="B11" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C11" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D11" t="s">
+        <v>660</v>
+      </c>
+      <c s="1" r="E11" t="s">
+        <v>1370</v>
+      </c>
+      <c s="1" r="F11" t="s">
+        <v>46</v>
+      </c>
+      <c s="1" r="G11" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="12">
+      <c s="1" r="A12" t="s">
+        <v>1371</v>
+      </c>
+      <c s="1" r="B12" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C12" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D12" t="s">
+        <v>684</v>
+      </c>
+      <c s="1" r="E12" t="s">
+        <v>889</v>
+      </c>
+      <c s="1" r="F12" t="s">
+        <v>51</v>
+      </c>
+      <c s="1" r="G12" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="13">
+      <c s="1" r="A13" t="s">
+        <v>1372</v>
+      </c>
+      <c s="1" r="B13" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C13" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D13" t="s">
         <v>638</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1" t="s">
+      <c s="1" r="E13" t="s">
+        <v>638</v>
+      </c>
+      <c s="1" r="F13" t="s">
         <v>115</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c s="1" r="G13" t="s">
         <v>639</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>640</v>
-      </c>
-      <c r="B3" s="1" t="s">
+    <row r="14">
+      <c s="1" r="A14" t="s">
+        <v>1373</v>
+      </c>
+      <c s="1" r="B14" t="s">
         <v>636</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c s="1" r="C14" t="s">
         <v>637</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c s="1" r="D14" t="s">
         <v>641</v>
       </c>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1" t="s">
+      <c s="1" r="E14" t="s">
+        <v>641</v>
+      </c>
+      <c s="1" r="F14" t="s">
         <v>115</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c s="1" r="G14" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>643</v>
-      </c>
-      <c r="B4" s="1" t="s">
+    <row r="15">
+      <c s="1" r="A15" t="s">
+        <v>1374</v>
+      </c>
+      <c s="1" r="B15" t="s">
         <v>636</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c s="1" r="C15" t="s">
         <v>637</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>645</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c s="1" r="D15" t="s">
+        <v>669</v>
+      </c>
+      <c s="1" r="E15" t="s">
+        <v>669</v>
+      </c>
+      <c s="1" r="F15" t="s">
+        <v>115</v>
+      </c>
+      <c s="1" r="G15" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="16">
+      <c s="1" r="A16" t="s">
+        <v>1375</v>
+      </c>
+      <c s="1" r="B16" t="s">
         <v>636</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c s="1" r="C16" t="s">
         <v>637</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>646</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>881</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c s="1" r="D16" t="s">
+        <v>678</v>
+      </c>
+      <c s="1" r="E16" t="s">
+        <v>678</v>
+      </c>
+      <c s="1" r="F16" t="s">
+        <v>115</v>
+      </c>
+      <c s="1" r="G16" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="17">
+      <c s="1" r="A17" t="s">
+        <v>1376</v>
+      </c>
+      <c s="1" r="B17" t="s">
+        <v>636</v>
+      </c>
+      <c s="1" r="C17" t="s">
+        <v>637</v>
+      </c>
+      <c s="1" r="D17" t="s">
+        <v>681</v>
+      </c>
+      <c s="1" r="E17" t="s">
+        <v>681</v>
+      </c>
+      <c s="1" r="F17" t="s">
         <v>647</v>
       </c>
-      <c r="G5" s="1" t="s">
-        <v>644</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>648</v>
-      </c>
-      <c r="B6" s="1" t="s">
+      <c s="1" r="G17" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="18">
+      <c s="1" r="A18" t="s">
+        <v>1377</v>
+      </c>
+      <c s="1" r="B18" t="s">
         <v>636</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c s="1" r="C18" t="s">
         <v>637</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>649</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>882</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>651</v>
-      </c>
-      <c r="B7" s="1" t="s">
+      <c s="1" r="D18" t="s">
+        <v>663</v>
+      </c>
+      <c s="1" r="E18" t="s">
+        <v>887</v>
+      </c>
+      <c s="1" r="F18" t="s">
+        <v>182</v>
+      </c>
+      <c s="1" r="G18" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="19">
+      <c s="1" r="A19" t="s">
+        <v>1378</v>
+      </c>
+      <c s="1" r="B19" t="s">
         <v>636</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c s="1" r="C19" t="s">
         <v>637</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1" t="s">
+      <c s="1" r="D19" t="s">
+        <v>657</v>
+      </c>
+      <c s="1" r="E19" t="s">
+        <v>886</v>
+      </c>
+      <c s="1" r="F19" t="s">
         <v>115</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>653</v>
-      </c>
-      <c r="B8" s="1" t="s">
+      <c s="1" r="G19" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="20">
+      <c s="1" r="A20" t="s">
+        <v>1379</v>
+      </c>
+      <c s="1" r="B20" t="s">
         <v>636</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c s="1" r="C20" t="s">
         <v>637</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c s="1" r="D20" t="s">
         <v>654</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c s="1" r="E20" t="s">
         <v>885</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c s="1" r="F20" t="s">
         <v>115</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c s="1" r="G20" t="s">
         <v>655</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>656</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>657</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>886</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>659</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>660</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>888</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>661</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>662</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>663</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>887</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>664</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>665</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>666</v>
-      </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>668</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>669</v>
-      </c>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>670</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>671</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>672</v>
-      </c>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>674</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>675</v>
-      </c>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>676</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
-        <v>677</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>678</v>
-      </c>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
-        <v>680</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>681</v>
-      </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1" t="s">
-        <v>647</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
-        <v>683</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>684</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>889</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>685</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
-        <v>686</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>687</v>
-      </c>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>688</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
-        <v>689</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>636</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>690</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>691</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removed unnecessary status badges
</commit_message>
<xml_diff>
--- a/translations/all-pages.xlsx
+++ b/translations/all-pages.xlsx
@@ -5033,7 +5033,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{AAE8341E-AA9D-44FB-828B-E8E7C198C373}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="14.5" ns3:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="27.6328125" bestFit="1" customWidth="1"/>
@@ -5410,7 +5410,7 @@
     </row>
     <row r="17">
       <c s="1" r="A17" t="s">
-        <v>1376</v>
+        <v>1377</v>
       </c>
       <c s="1" r="B17" t="s">
         <v>636</v>
@@ -5419,85 +5419,16 @@
         <v>637</v>
       </c>
       <c s="1" r="D17" t="s">
-        <v>681</v>
+        <v>663</v>
       </c>
       <c s="1" r="E17" t="s">
-        <v>681</v>
+        <v>887</v>
       </c>
       <c s="1" r="F17" t="s">
-        <v>647</v>
+        <v>182</v>
       </c>
       <c s="1" r="G17" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="18">
-      <c s="1" r="A18" t="s">
-        <v>1377</v>
-      </c>
-      <c s="1" r="B18" t="s">
-        <v>636</v>
-      </c>
-      <c s="1" r="C18" t="s">
-        <v>637</v>
-      </c>
-      <c s="1" r="D18" t="s">
-        <v>663</v>
-      </c>
-      <c s="1" r="E18" t="s">
-        <v>887</v>
-      </c>
-      <c s="1" r="F18" t="s">
-        <v>182</v>
-      </c>
-      <c s="1" r="G18" t="s">
         <v>664</v>
-      </c>
-    </row>
-    <row r="19">
-      <c s="1" r="A19" t="s">
-        <v>1378</v>
-      </c>
-      <c s="1" r="B19" t="s">
-        <v>636</v>
-      </c>
-      <c s="1" r="C19" t="s">
-        <v>637</v>
-      </c>
-      <c s="1" r="D19" t="s">
-        <v>657</v>
-      </c>
-      <c s="1" r="E19" t="s">
-        <v>886</v>
-      </c>
-      <c s="1" r="F19" t="s">
-        <v>115</v>
-      </c>
-      <c s="1" r="G19" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="20">
-      <c s="1" r="A20" t="s">
-        <v>1379</v>
-      </c>
-      <c s="1" r="B20" t="s">
-        <v>636</v>
-      </c>
-      <c s="1" r="C20" t="s">
-        <v>637</v>
-      </c>
-      <c s="1" r="D20" t="s">
-        <v>654</v>
-      </c>
-      <c s="1" r="E20" t="s">
-        <v>885</v>
-      </c>
-      <c s="1" r="F20" t="s">
-        <v>115</v>
-      </c>
-      <c s="1" r="G20" t="s">
-        <v>655</v>
       </c>
     </row>
   </sheetData>
@@ -5507,7 +5438,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{4418D199-425E-433A-A53F-5B6A45116917}">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr defaultRowHeight="14.5" ns3:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="4.453125" bestFit="1" customWidth="1"/>
@@ -6665,29 +6596,6 @@
       </c>
       <c s="1" r="G50" t="s">
         <v>738</v>
-      </c>
-    </row>
-    <row ns3:dyDescent="0.35" r="51">
-      <c s="1" r="A51" t="s">
-        <v>1096</v>
-      </c>
-      <c s="1" r="B51" t="s">
-        <v>693</v>
-      </c>
-      <c s="1" r="C51" t="s">
-        <v>694</v>
-      </c>
-      <c r="D51" t="s">
-        <v>781</v>
-      </c>
-      <c r="E51" t="s">
-        <v>781</v>
-      </c>
-      <c s="1" r="F51" t="s">
-        <v>115</v>
-      </c>
-      <c s="1" r="G51" t="s">
-        <v>782</v>
       </c>
     </row>
   </sheetData>

</xml_diff>